<commit_message>
km 사후 검정 update
</commit_message>
<xml_diff>
--- a/result/LOXL2_LUAD_Tables.xlsx
+++ b/result/LOXL2_LUAD_Tables.xlsx
@@ -3963,12 +3963,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>9.204</t>
+          <t>11.430</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.002</t>
+          <t>0.010</t>
         </is>
       </c>
     </row>
@@ -3990,12 +3990,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2.020</t>
+          <t>7.177</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.155</t>
+          <t>0.066</t>
         </is>
       </c>
     </row>

</xml_diff>